<commit_message>
updated data in ai_fallback and savehistory sheets by fakruddin
</commit_message>
<xml_diff>
--- a/src/test/resources/mytutorai_testcases.xlsx
+++ b/src/test/resources/mytutorai_testcases.xlsx
@@ -1,13 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2521732\Downloads\mytutorai\mytutorai\src\test\resources\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C67EA6E-11AE-4D7C-AC97-DCB9DC435BA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Save_History_Logout" sheetId="5" r:id="rId2"/>
+    <sheet name="AI_Fallback" sheetId="6" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -18,9 +26,212 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="66">
+  <si>
+    <t>fallback badge gone</t>
+  </si>
+  <si>
+    <t>AI-generated</t>
+  </si>
+  <si>
+    <t>Selenium implicit wait</t>
+  </si>
+  <si>
+    <t>Explain a concept</t>
+  </si>
+  <si>
+    <t>AI restored</t>
+  </si>
+  <si>
+    <t>full text copied; pasted text matches</t>
+  </si>
+  <si>
+    <t>Rule-based fallback</t>
+  </si>
+  <si>
+    <t>Selenium explicit wait</t>
+  </si>
+  <si>
+    <t>AI failing</t>
+  </si>
+  <si>
+    <t>Copy fallback answer</t>
+  </si>
+  <si>
+    <t>answer not empty</t>
+  </si>
+  <si>
+    <t>Learn through code</t>
+  </si>
+  <si>
+    <t>AI fails</t>
+  </si>
+  <si>
+    <t>Understand a use case</t>
+  </si>
+  <si>
+    <t>auto switch; no retry needed</t>
+  </si>
+  <si>
+    <t>Prepare for interview</t>
+  </si>
+  <si>
+    <t>AI timeout / no response</t>
+  </si>
+  <si>
+    <t>AI timeout</t>
+  </si>
+  <si>
+    <t>answer shown; no error page</t>
+  </si>
+  <si>
+    <t>AI failing (invalid key / service off)</t>
+  </si>
+  <si>
+    <t>no fallback badge</t>
+  </si>
+  <si>
+    <t>AI working</t>
+  </si>
+  <si>
+    <t>AI answer</t>
+  </si>
+  <si>
+    <t>expected</t>
+  </si>
+  <si>
+    <t>expectedSourceLabel</t>
+  </si>
+  <si>
+    <t>prompt</t>
+  </si>
+  <si>
+    <t>cardName</t>
+  </si>
+  <si>
+    <t>aiServiceState</t>
+  </si>
+  <si>
+    <t>scenario</t>
+  </si>
+  <si>
+    <t>login page shown; protected content not restored</t>
+  </si>
+  <si>
+    <t>Sign out, press Back, refresh</t>
+  </si>
+  <si>
+    <t>mtuser101</t>
+  </si>
+  <si>
+    <t>Secure logout</t>
+  </si>
+  <si>
+    <t>User 1 data not visible</t>
+  </si>
+  <si>
+    <t>Open History and Saved Content</t>
+  </si>
+  <si>
+    <t>mtuser102</t>
+  </si>
+  <si>
+    <t>Data isolation</t>
+  </si>
+  <si>
+    <t>saved content still present</t>
+  </si>
+  <si>
+    <t>Sign out, sign in, open Saved Content</t>
+  </si>
+  <si>
+    <t>Persistence after sign out</t>
+  </si>
+  <si>
+    <t>item removed; others remain</t>
+  </si>
+  <si>
+    <t>Remove</t>
+  </si>
+  <si>
+    <t>Explain implicit wait in Selenium with an example.</t>
+  </si>
+  <si>
+    <t>Remove saved item</t>
+  </si>
+  <si>
+    <t>History empty; Saved Content unchanged</t>
+  </si>
+  <si>
+    <t>Clear history</t>
+  </si>
+  <si>
+    <t>Clear History</t>
+  </si>
+  <si>
+    <t>prompt loaded on New Prompt page</t>
+  </si>
+  <si>
+    <t>History &gt; Use again</t>
+  </si>
+  <si>
+    <t>Explain Selenium locators with an example</t>
+  </si>
+  <si>
+    <t>Reuse prompt</t>
+  </si>
+  <si>
+    <t>listed above entry 1 (latest first)</t>
+  </si>
+  <si>
+    <t>Generate, open History</t>
+  </si>
+  <si>
+    <t>What is explicit wait in Selenium?</t>
+  </si>
+  <si>
+    <t>History entry 2</t>
+  </si>
+  <si>
+    <t>entry listed with topic, preview, source, date-time</t>
+  </si>
+  <si>
+    <t>History entry 1</t>
+  </si>
+  <si>
+    <t>no crash; duplicate handled consistently</t>
+  </si>
+  <si>
+    <t>Click Save twice</t>
+  </si>
+  <si>
+    <t>Save same answer twice</t>
+  </si>
+  <si>
+    <t>appears in Saved Content</t>
+  </si>
+  <si>
+    <t>Generate, click Save</t>
+  </si>
+  <si>
+    <t>Explain explicit wait in Selenium in simple terms with an example.</t>
+  </si>
+  <si>
+    <t>Save answer</t>
+  </si>
+  <si>
+    <t>action</t>
+  </si>
+  <si>
+    <t>userId</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -28,16 +239,31 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +271,33 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFBFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +577,444 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1529D749-C4C3-46A6-997E-D771F5027779}">
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="50" customWidth="1"/>
+    <col min="4" max="4" width="39" customWidth="1"/>
+    <col min="5" max="5" width="50" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="25" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="1"/>
+      <c r="D9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E706A60-B232-4274-A9C3-6268C306787A}">
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="1"/>
+    <col min="2" max="2" width="40" customWidth="1"/>
+    <col min="3" max="3" width="23" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="5" max="5" width="21" customWidth="1"/>
+    <col min="6" max="6" width="39" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Updated data in promptknowledge by Venkata Ganesh
</commit_message>
<xml_diff>
--- a/src/test/resources/mytutorai_testcases.xlsx
+++ b/src/test/resources/mytutorai_testcases.xlsx
@@ -5,15 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2521732\Downloads\mytutorai\mytutorai\src\test\resources\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2521765\Downloads\mytutorai\src\test\resources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C67EA6E-11AE-4D7C-AC97-DCB9DC435BA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{137DBB80-A7C3-48F6-9D6B-4A1F6C1311B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Prompt_Knowledge" sheetId="7" r:id="rId1"/>
     <sheet name="Save_History_Logout" sheetId="5" r:id="rId2"/>
     <sheet name="AI_Fallback" sheetId="6" r:id="rId3"/>
   </sheets>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="92">
   <si>
     <t>fallback badge gone</t>
   </si>
@@ -225,6 +225,84 @@
   </si>
   <si>
     <t>userId</t>
+  </si>
+  <si>
+    <t>Requested topic not found in the knowledge repository.</t>
+  </si>
+  <si>
+    <t>Explain quantum computing qubits in simple terms.</t>
+  </si>
+  <si>
+    <t>Topic not in repository</t>
+  </si>
+  <si>
+    <t>no script runs; page does not break</t>
+  </si>
+  <si>
+    <t>What is @#$%^&amp;*() &lt;script&gt;alert(1)&lt;/script&gt; in Selenium wait?</t>
+  </si>
+  <si>
+    <t>Special characters</t>
+  </si>
+  <si>
+    <t>no crash; response or message shown</t>
+  </si>
+  <si>
+    <t>selenium-notes.txt</t>
+  </si>
+  <si>
+    <t>I am preparing for a QA automation interview and want to understand how Selenium handles waiting for elements on dynamic pages, including explicit, implicit and fluent wait, when to use each and common mistakes. I am preparing for a QA automation interview and want to understand how Selenium handles waiting for elements on dynamic pages, including explicit, implicit and fluent wait, when to use each and common mistakes. I am preparing for a QA automation interview and want to understand how Selenium handles waiting for elements on dynamic pages, including explicit, implicit and fluent wait, when to use each and common mistakes. I am preparing for a QA automation interview and want to understand how Selenium handles waiting for elements on dynamic pages, including explicit, implicit and fluent wait, when to use each and common mistakes. I am preparing for a QA automation interview and want to understand how Selenium handles waiting for elements on dynamic pages, including explicit, implicit and fluent wait, when to use each and common mistakes. I am preparing for a QA automation interview and want to understand how Selenium handles waiting for elements on dynamic pages, including explicit, implicit and fluent wait, when to use each and common mistakes. I am preparing for a QA automation interview and want to understand how Selenium handles waiting for elements on dynamic pages, including explicit, implicit and fluent wait, when to use each and common mistakes. I am preparing for a QA automation interview and want to understand how Selenium handles waiting for elements on dynamic pages, including explicit, implicit and fluent wait, when to use each and common mistakes.</t>
+  </si>
+  <si>
+    <t>Very long prompt (~300 words)</t>
+  </si>
+  <si>
+    <t>relevant response shown</t>
+  </si>
+  <si>
+    <t>Selenium wait</t>
+  </si>
+  <si>
+    <t>Keyword only</t>
+  </si>
+  <si>
+    <t>Give an example of explicit wait.</t>
+  </si>
+  <si>
+    <t>Instruction format</t>
+  </si>
+  <si>
+    <t>Question format</t>
+  </si>
+  <si>
+    <t>generation starts like Generate answer</t>
+  </si>
+  <si>
+    <t>Ctrl + Enter</t>
+  </si>
+  <si>
+    <t>treated as empty; no answer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">     </t>
+  </si>
+  <si>
+    <t>Whitespace only</t>
+  </si>
+  <si>
+    <t>no answer; submission blocked</t>
+  </si>
+  <si>
+    <t>Empty prompt</t>
+  </si>
+  <si>
+    <t>answer shown; topic Selenium</t>
+  </si>
+  <si>
+    <t>Valid prompt</t>
+  </si>
+  <si>
+    <t>expectedKnowledgeSource</t>
   </si>
 </sst>
 </file>
@@ -577,11 +655,162 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{496D60FB-5AAB-4541-B36A-823F5BBF1491}">
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <cols>
+    <col min="1" max="1" width="31" customWidth="1"/>
+    <col min="2" max="2" width="50" customWidth="1"/>
+    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="4" max="4" width="50" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+      <c r="A5" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="375" x14ac:dyDescent="0.35">
+      <c r="A9" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="25" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 

</xml_diff>